<commit_message>
Update INARA Beta 12 WOK 2026-10-03 09:31:18
</commit_message>
<xml_diff>
--- a/beta_12wok/detail_odp_black_special_value.xlsx
+++ b/beta_12wok/detail_odp_black_special_value.xlsx
@@ -211,10 +211,10 @@
     <t>LOMBOK</t>
   </si>
   <si>
-    <t>KUPANG ROTE</t>
-  </si>
-  <si>
-    <t>BALI TENGAH</t>
+    <t>KUPANG ROTE - MALAKA TIMTIM BELU</t>
+  </si>
+  <si>
+    <t>BALI TENGAH 2</t>
   </si>
   <si>
     <t>LOMBOK 1</t>

</xml_diff>

<commit_message>
Update INARA Beta 12 WOK 2026-10-03 10:11:29
</commit_message>
<xml_diff>
--- a/beta_12wok/detail_odp_black_special_value.xlsx
+++ b/beta_12wok/detail_odp_black_special_value.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="113">
   <si>
     <t>ODP</t>
   </si>
@@ -211,16 +211,10 @@
     <t>LOMBOK</t>
   </si>
   <si>
-    <t>KUPANG ROTE - MALAKA TIMTIM BELU</t>
-  </si>
-  <si>
-    <t>BALI TENGAH 2</t>
-  </si>
-  <si>
-    <t>LOMBOK 1</t>
-  </si>
-  <si>
-    <t>LOMBOK 2</t>
+    <t>KUPANG ROTE</t>
+  </si>
+  <si>
+    <t>BALI TENGAH</t>
   </si>
   <si>
     <t>TABANAN</t>
@@ -786,13 +780,13 @@
         <v>63</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="I2">
         <v>-8.508568474</v>
@@ -801,7 +795,7 @@
         <v>115.1998034</v>
       </c>
       <c r="K2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L2">
         <v>2</v>
@@ -819,7 +813,7 @@
         <v>1</v>
       </c>
       <c r="Q2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -836,13 +830,13 @@
         <v>63</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I3">
         <v>-8.526441949000001</v>
@@ -851,7 +845,7 @@
         <v>115.1364796</v>
       </c>
       <c r="K3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L3">
         <v>0</v>
@@ -869,7 +863,7 @@
         <v>1</v>
       </c>
       <c r="Q3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -885,17 +879,14 @@
       <c r="D4" t="s">
         <v>64</v>
       </c>
-      <c r="E4" t="s">
-        <v>67</v>
-      </c>
       <c r="F4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="I4">
         <v>-8.602909052999999</v>
@@ -904,7 +895,7 @@
         <v>116.1536542</v>
       </c>
       <c r="K4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L4">
         <v>1</v>
@@ -922,7 +913,7 @@
         <v>1</v>
       </c>
       <c r="Q4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -938,17 +929,14 @@
       <c r="D5" t="s">
         <v>64</v>
       </c>
-      <c r="E5" t="s">
-        <v>67</v>
-      </c>
       <c r="F5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I5">
         <v>-8.602367258999999</v>
@@ -957,7 +945,7 @@
         <v>116.1430562</v>
       </c>
       <c r="K5" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -975,7 +963,7 @@
         <v>1</v>
       </c>
       <c r="Q5" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -991,17 +979,14 @@
       <c r="D6" t="s">
         <v>64</v>
       </c>
-      <c r="E6" t="s">
-        <v>67</v>
-      </c>
       <c r="F6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H6" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I6">
         <v>-8.603221198</v>
@@ -1010,7 +995,7 @@
         <v>116.143717</v>
       </c>
       <c r="K6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L6">
         <v>0</v>
@@ -1028,7 +1013,7 @@
         <v>1</v>
       </c>
       <c r="Q6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -1044,17 +1029,14 @@
       <c r="D7" t="s">
         <v>64</v>
       </c>
-      <c r="E7" t="s">
-        <v>67</v>
-      </c>
       <c r="F7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="I7">
         <v>-8.599239378</v>
@@ -1063,7 +1045,7 @@
         <v>116.1329936</v>
       </c>
       <c r="K7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -1081,7 +1063,7 @@
         <v>1</v>
       </c>
       <c r="Q7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1097,17 +1079,14 @@
       <c r="D8" t="s">
         <v>64</v>
       </c>
-      <c r="E8" t="s">
-        <v>67</v>
-      </c>
       <c r="F8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H8" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="I8">
         <v>-8.627093541000001</v>
@@ -1116,7 +1095,7 @@
         <v>116.1328874</v>
       </c>
       <c r="K8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L8">
         <v>0</v>
@@ -1134,7 +1113,7 @@
         <v>1</v>
       </c>
       <c r="Q8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -1150,17 +1129,14 @@
       <c r="D9" t="s">
         <v>64</v>
       </c>
-      <c r="E9" t="s">
-        <v>67</v>
-      </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="I9">
         <v>-8.627538016000001</v>
@@ -1169,7 +1145,7 @@
         <v>116.1327942</v>
       </c>
       <c r="K9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L9">
         <v>0</v>
@@ -1187,7 +1163,7 @@
         <v>1</v>
       </c>
       <c r="Q9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1203,17 +1179,14 @@
       <c r="D10" t="s">
         <v>64</v>
       </c>
-      <c r="E10" t="s">
-        <v>67</v>
-      </c>
       <c r="F10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="I10">
         <v>-8.358494758999999</v>
@@ -1222,7 +1195,7 @@
         <v>116.1495849</v>
       </c>
       <c r="K10" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L10">
         <v>0</v>
@@ -1240,7 +1213,7 @@
         <v>1</v>
       </c>
       <c r="Q10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -1256,17 +1229,14 @@
       <c r="D11" t="s">
         <v>64</v>
       </c>
-      <c r="E11" t="s">
-        <v>67</v>
-      </c>
       <c r="F11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G11" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H11" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="I11">
         <v>-8.358866183</v>
@@ -1275,7 +1245,7 @@
         <v>116.1487853</v>
       </c>
       <c r="K11" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L11">
         <v>0</v>
@@ -1293,7 +1263,7 @@
         <v>1</v>
       </c>
       <c r="Q11" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -1309,17 +1279,14 @@
       <c r="D12" t="s">
         <v>64</v>
       </c>
-      <c r="E12" t="s">
-        <v>67</v>
-      </c>
       <c r="F12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H12" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I12">
         <v>-8.34948075</v>
@@ -1328,7 +1295,7 @@
         <v>116.1686008</v>
       </c>
       <c r="K12" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -1346,7 +1313,7 @@
         <v>1</v>
       </c>
       <c r="Q12" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1362,17 +1329,14 @@
       <c r="D13" t="s">
         <v>64</v>
       </c>
-      <c r="E13" t="s">
-        <v>67</v>
-      </c>
       <c r="F13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G13" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H13" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I13">
         <v>-8.347617261</v>
@@ -1381,7 +1345,7 @@
         <v>116.1690833</v>
       </c>
       <c r="K13" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L13">
         <v>1</v>
@@ -1399,7 +1363,7 @@
         <v>1</v>
       </c>
       <c r="Q13" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1415,17 +1379,14 @@
       <c r="D14" t="s">
         <v>64</v>
       </c>
-      <c r="E14" t="s">
-        <v>68</v>
-      </c>
       <c r="F14" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G14" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H14" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I14">
         <v>-8.587127515000001</v>
@@ -1434,7 +1395,7 @@
         <v>116.3125604</v>
       </c>
       <c r="K14" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L14">
         <v>0</v>
@@ -1452,7 +1413,7 @@
         <v>1</v>
       </c>
       <c r="Q14" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1468,17 +1429,14 @@
       <c r="D15" t="s">
         <v>64</v>
       </c>
-      <c r="E15" t="s">
-        <v>68</v>
-      </c>
       <c r="F15" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G15" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H15" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I15">
         <v>-8.586417143</v>
@@ -1487,7 +1445,7 @@
         <v>116.3120566</v>
       </c>
       <c r="K15" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L15">
         <v>0</v>
@@ -1505,7 +1463,7 @@
         <v>1</v>
       </c>
       <c r="Q15" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -1521,17 +1479,14 @@
       <c r="D16" t="s">
         <v>64</v>
       </c>
-      <c r="E16" t="s">
-        <v>68</v>
-      </c>
       <c r="F16" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G16" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H16" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I16">
         <v>-8.586269807000001</v>
@@ -1540,7 +1495,7 @@
         <v>116.3106078</v>
       </c>
       <c r="K16" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L16">
         <v>0</v>
@@ -1558,7 +1513,7 @@
         <v>1</v>
       </c>
       <c r="Q16" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="17" spans="1:17">
@@ -1574,17 +1529,14 @@
       <c r="D17" t="s">
         <v>64</v>
       </c>
-      <c r="E17" t="s">
-        <v>68</v>
-      </c>
       <c r="F17" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H17" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I17">
         <v>-8.586482159999999</v>
@@ -1593,7 +1545,7 @@
         <v>116.3092842</v>
       </c>
       <c r="K17" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L17">
         <v>0</v>
@@ -1611,7 +1563,7 @@
         <v>1</v>
       </c>
       <c r="Q17" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:17">
@@ -1627,17 +1579,14 @@
       <c r="D18" t="s">
         <v>64</v>
       </c>
-      <c r="E18" t="s">
-        <v>68</v>
-      </c>
       <c r="F18" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G18" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H18" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I18">
         <v>-8.587142588000001</v>
@@ -1646,7 +1595,7 @@
         <v>116.3086122</v>
       </c>
       <c r="K18" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L18">
         <v>0</v>
@@ -1664,7 +1613,7 @@
         <v>1</v>
       </c>
       <c r="Q18" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:17">
@@ -1680,17 +1629,14 @@
       <c r="D19" t="s">
         <v>64</v>
       </c>
-      <c r="E19" t="s">
-        <v>68</v>
-      </c>
       <c r="F19" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H19" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I19">
         <v>-8.587113602000001</v>
@@ -1699,7 +1645,7 @@
         <v>116.3080444</v>
       </c>
       <c r="K19" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L19">
         <v>0</v>
@@ -1717,7 +1663,7 @@
         <v>1</v>
       </c>
       <c r="Q19" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:17">
@@ -1733,17 +1679,14 @@
       <c r="D20" t="s">
         <v>64</v>
       </c>
-      <c r="E20" t="s">
-        <v>68</v>
-      </c>
       <c r="F20" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G20" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H20" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I20">
         <v>-8.587634986999999</v>
@@ -1752,7 +1695,7 @@
         <v>116.307917</v>
       </c>
       <c r="K20" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L20">
         <v>0</v>
@@ -1770,7 +1713,7 @@
         <v>1</v>
       </c>
       <c r="Q20" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:17">
@@ -1786,17 +1729,14 @@
       <c r="D21" t="s">
         <v>64</v>
       </c>
-      <c r="E21" t="s">
-        <v>68</v>
-      </c>
       <c r="F21" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G21" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H21" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I21">
         <v>-8.589391066999999</v>
@@ -1805,7 +1745,7 @@
         <v>116.3103036</v>
       </c>
       <c r="K21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L21">
         <v>0</v>
@@ -1823,7 +1763,7 @@
         <v>1</v>
       </c>
       <c r="Q21" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:17">
@@ -1839,17 +1779,14 @@
       <c r="D22" t="s">
         <v>64</v>
       </c>
-      <c r="E22" t="s">
-        <v>68</v>
-      </c>
       <c r="F22" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G22" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H22" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I22">
         <v>-8.589132962000001</v>
@@ -1858,7 +1795,7 @@
         <v>116.3069518</v>
       </c>
       <c r="K22" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L22">
         <v>0</v>
@@ -1876,7 +1813,7 @@
         <v>1</v>
       </c>
       <c r="Q22" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23" spans="1:17">
@@ -1892,17 +1829,14 @@
       <c r="D23" t="s">
         <v>64</v>
       </c>
-      <c r="E23" t="s">
-        <v>68</v>
-      </c>
       <c r="F23" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G23" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H23" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I23">
         <v>-8.589509</v>
@@ -1911,7 +1845,7 @@
         <v>116.3057</v>
       </c>
       <c r="K23" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L23">
         <v>1</v>
@@ -1929,7 +1863,7 @@
         <v>1</v>
       </c>
       <c r="Q23" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="24" spans="1:17">
@@ -1945,17 +1879,14 @@
       <c r="D24" t="s">
         <v>64</v>
       </c>
-      <c r="E24" t="s">
-        <v>68</v>
-      </c>
       <c r="F24" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G24" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="H24" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="I24">
         <v>-8.588048634</v>
@@ -1964,7 +1895,7 @@
         <v>116.3472497</v>
       </c>
       <c r="K24" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L24">
         <v>0</v>
@@ -1982,7 +1913,7 @@
         <v>1</v>
       </c>
       <c r="Q24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="25" spans="1:17">
@@ -1998,17 +1929,14 @@
       <c r="D25" t="s">
         <v>64</v>
       </c>
-      <c r="E25" t="s">
-        <v>68</v>
-      </c>
       <c r="F25" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G25" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H25" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I25">
         <v>-8.587743615999999</v>
@@ -2017,7 +1945,7 @@
         <v>116.3199546</v>
       </c>
       <c r="K25" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="L25">
         <v>5</v>
@@ -2035,7 +1963,7 @@
         <v>1</v>
       </c>
       <c r="Q25" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="26" spans="1:17">
@@ -2051,17 +1979,14 @@
       <c r="D26" t="s">
         <v>64</v>
       </c>
-      <c r="E26" t="s">
-        <v>68</v>
-      </c>
       <c r="F26" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G26" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H26" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I26">
         <v>-8.589379918000001</v>
@@ -2070,7 +1995,7 @@
         <v>116.3183431</v>
       </c>
       <c r="K26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L26">
         <v>0</v>
@@ -2088,7 +2013,7 @@
         <v>1</v>
       </c>
       <c r="Q26" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="27" spans="1:17">
@@ -2104,17 +2029,14 @@
       <c r="D27" t="s">
         <v>64</v>
       </c>
-      <c r="E27" t="s">
-        <v>68</v>
-      </c>
       <c r="F27" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G27" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H27" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="I27">
         <v>-8.589138937</v>
@@ -2123,7 +2045,7 @@
         <v>116.307804</v>
       </c>
       <c r="K27" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L27">
         <v>0</v>
@@ -2141,7 +2063,7 @@
         <v>1</v>
       </c>
       <c r="Q27" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28" spans="1:17">
@@ -2157,17 +2079,14 @@
       <c r="D28" t="s">
         <v>64</v>
       </c>
-      <c r="E28" t="s">
-        <v>68</v>
-      </c>
       <c r="F28" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G28" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="H28" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I28">
         <v>-8.592968228</v>
@@ -2176,7 +2095,7 @@
         <v>116.2928783</v>
       </c>
       <c r="K28" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L28">
         <v>1</v>
@@ -2194,7 +2113,7 @@
         <v>1</v>
       </c>
       <c r="Q28" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" spans="1:17">
@@ -2210,17 +2129,14 @@
       <c r="D29" t="s">
         <v>64</v>
       </c>
-      <c r="E29" t="s">
-        <v>68</v>
-      </c>
       <c r="F29" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G29" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="H29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I29">
         <v>-8.592359</v>
@@ -2229,7 +2145,7 @@
         <v>116.2898168</v>
       </c>
       <c r="K29" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L29">
         <v>0</v>
@@ -2247,7 +2163,7 @@
         <v>1</v>
       </c>
       <c r="Q29" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:17">
@@ -2263,17 +2179,14 @@
       <c r="D30" t="s">
         <v>64</v>
       </c>
-      <c r="E30" t="s">
-        <v>68</v>
-      </c>
       <c r="F30" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G30" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H30" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="I30">
         <v>-8.616699897</v>
@@ -2282,7 +2195,7 @@
         <v>116.3165238</v>
       </c>
       <c r="K30" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L30">
         <v>1</v>
@@ -2300,7 +2213,7 @@
         <v>1</v>
       </c>
       <c r="Q30" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="31" spans="1:17">
@@ -2316,17 +2229,14 @@
       <c r="D31" t="s">
         <v>64</v>
       </c>
-      <c r="E31" t="s">
-        <v>68</v>
-      </c>
       <c r="F31" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G31" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H31" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="I31">
         <v>-8.801802138999999</v>
@@ -2335,7 +2245,7 @@
         <v>116.23624</v>
       </c>
       <c r="K31" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L31">
         <v>0</v>
@@ -2353,7 +2263,7 @@
         <v>1</v>
       </c>
       <c r="Q31" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="32" spans="1:17">
@@ -2369,17 +2279,14 @@
       <c r="D32" t="s">
         <v>64</v>
       </c>
-      <c r="E32" t="s">
-        <v>68</v>
-      </c>
       <c r="F32" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G32" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H32" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="I32">
         <v>-8.707284808000001</v>
@@ -2388,7 +2295,7 @@
         <v>116.2666262</v>
       </c>
       <c r="K32" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L32">
         <v>0</v>
@@ -2406,7 +2313,7 @@
         <v>1</v>
       </c>
       <c r="Q32" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="33" spans="1:17">
@@ -2423,13 +2330,13 @@
         <v>65</v>
       </c>
       <c r="F33" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G33" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H33" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I33">
         <v>-10.15818294</v>
@@ -2438,7 +2345,7 @@
         <v>123.6654479</v>
       </c>
       <c r="K33" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L33">
         <v>2</v>
@@ -2456,7 +2363,7 @@
         <v>1</v>
       </c>
       <c r="Q33" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="34" spans="1:17">
@@ -2473,13 +2380,13 @@
         <v>65</v>
       </c>
       <c r="F34" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G34" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H34" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I34">
         <v>-10.15797653</v>
@@ -2488,7 +2395,7 @@
         <v>123.6662125</v>
       </c>
       <c r="K34" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L34">
         <v>0</v>
@@ -2506,7 +2413,7 @@
         <v>1</v>
       </c>
       <c r="Q34" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="35" spans="1:17">
@@ -2523,13 +2430,13 @@
         <v>66</v>
       </c>
       <c r="F35" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G35" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H35" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="I35">
         <v>-8.699028999999999</v>
@@ -2538,7 +2445,7 @@
         <v>115.2086979</v>
       </c>
       <c r="K35" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L35">
         <v>1</v>
@@ -2556,7 +2463,7 @@
         <v>1</v>
       </c>
       <c r="Q35" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="36" spans="1:17">
@@ -2573,13 +2480,13 @@
         <v>63</v>
       </c>
       <c r="F36" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G36" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H36" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I36">
         <v>-8.369822170999999</v>
@@ -2588,7 +2495,7 @@
         <v>115.1925405</v>
       </c>
       <c r="K36" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L36">
         <v>2</v>
@@ -2606,7 +2513,7 @@
         <v>1</v>
       </c>
       <c r="Q36" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="37" spans="1:17">
@@ -2623,13 +2530,13 @@
         <v>63</v>
       </c>
       <c r="F37" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G37" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H37" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I37">
         <v>-8.36708297</v>
@@ -2638,7 +2545,7 @@
         <v>115.1921949</v>
       </c>
       <c r="K37" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L37">
         <v>1</v>
@@ -2656,7 +2563,7 @@
         <v>1</v>
       </c>
       <c r="Q37" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="38" spans="1:17">
@@ -2673,13 +2580,13 @@
         <v>63</v>
       </c>
       <c r="F38" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G38" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H38" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="I38">
         <v>-8.364740604</v>
@@ -2688,7 +2595,7 @@
         <v>115.1918556</v>
       </c>
       <c r="K38" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L38">
         <v>2</v>
@@ -2706,7 +2613,7 @@
         <v>1</v>
       </c>
       <c r="Q38" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39" spans="1:17">
@@ -2723,13 +2630,13 @@
         <v>63</v>
       </c>
       <c r="F39" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G39" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H39" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I39">
         <v>-8.382409832</v>
@@ -2738,7 +2645,7 @@
         <v>115.1953139</v>
       </c>
       <c r="K39" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L39">
         <v>2</v>
@@ -2756,7 +2663,7 @@
         <v>1</v>
       </c>
       <c r="Q39" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="40" spans="1:17">
@@ -2773,13 +2680,13 @@
         <v>63</v>
       </c>
       <c r="F40" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G40" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H40" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I40">
         <v>-8.392661041</v>
@@ -2788,7 +2695,7 @@
         <v>115.1955531</v>
       </c>
       <c r="K40" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L40">
         <v>0</v>
@@ -2806,7 +2713,7 @@
         <v>1</v>
       </c>
       <c r="Q40" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="41" spans="1:17">
@@ -2823,13 +2730,13 @@
         <v>63</v>
       </c>
       <c r="F41" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G41" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H41" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I41">
         <v>-8.394319465000001</v>
@@ -2838,7 +2745,7 @@
         <v>115.1955146</v>
       </c>
       <c r="K41" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L41">
         <v>1</v>
@@ -2856,7 +2763,7 @@
         <v>1</v>
       </c>
       <c r="Q41" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="42" spans="1:17">
@@ -2873,13 +2780,13 @@
         <v>63</v>
       </c>
       <c r="F42" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G42" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H42" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I42">
         <v>-8.401367157999999</v>
@@ -2888,7 +2795,7 @@
         <v>115.1964986</v>
       </c>
       <c r="K42" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -2906,7 +2813,7 @@
         <v>1</v>
       </c>
       <c r="Q42" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="43" spans="1:17">
@@ -2923,13 +2830,13 @@
         <v>63</v>
       </c>
       <c r="F43" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G43" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H43" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="I43">
         <v>-8.404993971</v>
@@ -2938,7 +2845,7 @@
         <v>115.1969283</v>
       </c>
       <c r="K43" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L43">
         <v>1</v>
@@ -2956,7 +2863,7 @@
         <v>1</v>
       </c>
       <c r="Q43" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update INARA Beta 12 WOK 2026-10-04 20:47:31
</commit_message>
<xml_diff>
--- a/beta_12wok/detail_odp_black_special_value.xlsx
+++ b/beta_12wok/detail_odp_black_special_value.xlsx
@@ -807,10 +807,10 @@
         <v>2</v>
       </c>
       <c r="O2">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="s">
         <v>112</v>
@@ -857,10 +857,10 @@
         <v>0</v>
       </c>
       <c r="O3">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="P3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q3" t="s">
         <v>112</v>
@@ -907,10 +907,10 @@
         <v>1</v>
       </c>
       <c r="O4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="s">
         <v>112</v>
@@ -957,10 +957,10 @@
         <v>0</v>
       </c>
       <c r="O5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="s">
         <v>112</v>
@@ -1007,10 +1007,10 @@
         <v>0</v>
       </c>
       <c r="O6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="s">
         <v>112</v>
@@ -1057,10 +1057,10 @@
         <v>0</v>
       </c>
       <c r="O7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="s">
         <v>112</v>
@@ -1107,10 +1107,10 @@
         <v>0</v>
       </c>
       <c r="O8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="s">
         <v>112</v>
@@ -1157,10 +1157,10 @@
         <v>0</v>
       </c>
       <c r="O9">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="s">
         <v>112</v>
@@ -1207,10 +1207,10 @@
         <v>0</v>
       </c>
       <c r="O10">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="s">
         <v>112</v>
@@ -1257,10 +1257,10 @@
         <v>0</v>
       </c>
       <c r="O11">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q11" t="s">
         <v>112</v>
@@ -1307,10 +1307,10 @@
         <v>0</v>
       </c>
       <c r="O12">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="s">
         <v>112</v>
@@ -1357,10 +1357,10 @@
         <v>1</v>
       </c>
       <c r="O13">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="s">
         <v>112</v>
@@ -1407,10 +1407,10 @@
         <v>0</v>
       </c>
       <c r="O14">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q14" t="s">
         <v>112</v>
@@ -1457,10 +1457,10 @@
         <v>0</v>
       </c>
       <c r="O15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q15" t="s">
         <v>112</v>
@@ -1507,10 +1507,10 @@
         <v>0</v>
       </c>
       <c r="O16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q16" t="s">
         <v>112</v>
@@ -1557,10 +1557,10 @@
         <v>0</v>
       </c>
       <c r="O17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q17" t="s">
         <v>112</v>
@@ -1607,10 +1607,10 @@
         <v>0</v>
       </c>
       <c r="O18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="s">
         <v>112</v>
@@ -1657,10 +1657,10 @@
         <v>0</v>
       </c>
       <c r="O19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q19" t="s">
         <v>112</v>
@@ -1707,10 +1707,10 @@
         <v>0</v>
       </c>
       <c r="O20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q20" t="s">
         <v>112</v>
@@ -1757,10 +1757,10 @@
         <v>0</v>
       </c>
       <c r="O21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q21" t="s">
         <v>112</v>
@@ -1807,10 +1807,10 @@
         <v>0</v>
       </c>
       <c r="O22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q22" t="s">
         <v>112</v>
@@ -1857,10 +1857,10 @@
         <v>1</v>
       </c>
       <c r="O23">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q23" t="s">
         <v>112</v>
@@ -1907,10 +1907,10 @@
         <v>0</v>
       </c>
       <c r="O24">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q24" t="s">
         <v>112</v>
@@ -1957,10 +1957,10 @@
         <v>1</v>
       </c>
       <c r="O25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q25" t="s">
         <v>112</v>
@@ -2007,10 +2007,10 @@
         <v>0</v>
       </c>
       <c r="O26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q26" t="s">
         <v>112</v>
@@ -2057,10 +2057,10 @@
         <v>0</v>
       </c>
       <c r="O27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q27" t="s">
         <v>112</v>
@@ -2107,10 +2107,10 @@
         <v>1</v>
       </c>
       <c r="O28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q28" t="s">
         <v>112</v>
@@ -2157,10 +2157,10 @@
         <v>0</v>
       </c>
       <c r="O29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q29" t="s">
         <v>112</v>
@@ -2207,10 +2207,10 @@
         <v>1</v>
       </c>
       <c r="O30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q30" t="s">
         <v>112</v>
@@ -2257,10 +2257,10 @@
         <v>0</v>
       </c>
       <c r="O31">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q31" t="s">
         <v>112</v>
@@ -2307,10 +2307,10 @@
         <v>0</v>
       </c>
       <c r="O32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q32" t="s">
         <v>112</v>
@@ -2357,10 +2357,10 @@
         <v>0</v>
       </c>
       <c r="O33">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="P33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q33" t="s">
         <v>112</v>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="O34">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="P34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q34" t="s">
         <v>112</v>
@@ -2457,10 +2457,10 @@
         <v>1</v>
       </c>
       <c r="O35">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q35" t="s">
         <v>112</v>
@@ -2507,10 +2507,10 @@
         <v>1</v>
       </c>
       <c r="O36">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="P36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q36" t="s">
         <v>112</v>
@@ -2557,10 +2557,10 @@
         <v>1</v>
       </c>
       <c r="O37">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q37" t="s">
         <v>112</v>
@@ -2607,10 +2607,10 @@
         <v>2</v>
       </c>
       <c r="O38">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q38" t="s">
         <v>112</v>
@@ -2657,10 +2657,10 @@
         <v>1</v>
       </c>
       <c r="O39">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q39" t="s">
         <v>112</v>
@@ -2707,10 +2707,10 @@
         <v>0</v>
       </c>
       <c r="O40">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="P40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q40" t="s">
         <v>112</v>
@@ -2757,10 +2757,10 @@
         <v>1</v>
       </c>
       <c r="O41">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="P41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q41" t="s">
         <v>112</v>
@@ -2807,10 +2807,10 @@
         <v>3</v>
       </c>
       <c r="O42">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="P42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q42" t="s">
         <v>112</v>
@@ -2857,10 +2857,10 @@
         <v>1</v>
       </c>
       <c r="O43">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q43" t="s">
         <v>112</v>

</xml_diff>

<commit_message>
Update INARA Beta 12 WOK 2026-10-08 15:10:16
</commit_message>
<xml_diff>
--- a/beta_12wok/detail_odp_black_special_value.xlsx
+++ b/beta_12wok/detail_odp_black_special_value.xlsx
@@ -2848,13 +2848,13 @@
         <v>109</v>
       </c>
       <c r="L43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M43">
         <v>0</v>
       </c>
       <c r="N43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O43">
         <v>0</v>

</xml_diff>

<commit_message>
Update INARA Beta 12 WOK 2026-10-14 07:39:28
</commit_message>
<xml_diff>
--- a/beta_12wok/detail_odp_black_special_value.xlsx
+++ b/beta_12wok/detail_odp_black_special_value.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="114">
   <si>
     <t>ODP</t>
   </si>
@@ -347,6 +347,9 @@
   </si>
   <si>
     <t>BLACK</t>
+  </si>
+  <si>
+    <t>RED</t>
   </si>
   <si>
     <t>YELLOW</t>
@@ -813,7 +816,7 @@
         <v>0</v>
       </c>
       <c r="Q2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -863,7 +866,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -913,7 +916,7 @@
         <v>0</v>
       </c>
       <c r="Q4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -963,7 +966,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -1013,7 +1016,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -1063,7 +1066,7 @@
         <v>0</v>
       </c>
       <c r="Q7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1113,7 +1116,7 @@
         <v>0</v>
       </c>
       <c r="Q8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -1163,7 +1166,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1213,7 +1216,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -1263,7 +1266,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -1313,7 +1316,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1363,7 +1366,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1413,7 +1416,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1463,7 +1466,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -1513,7 +1516,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="17" spans="1:17">
@@ -1563,7 +1566,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" spans="1:17">
@@ -1613,7 +1616,7 @@
         <v>0</v>
       </c>
       <c r="Q18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:17">
@@ -1663,7 +1666,7 @@
         <v>0</v>
       </c>
       <c r="Q19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:17">
@@ -1713,7 +1716,7 @@
         <v>0</v>
       </c>
       <c r="Q20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:17">
@@ -1763,7 +1766,7 @@
         <v>0</v>
       </c>
       <c r="Q21" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:17">
@@ -1813,7 +1816,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="23" spans="1:17">
@@ -1863,7 +1866,7 @@
         <v>0</v>
       </c>
       <c r="Q23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="24" spans="1:17">
@@ -1913,7 +1916,7 @@
         <v>0</v>
       </c>
       <c r="Q24" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="25" spans="1:17">
@@ -1948,13 +1951,13 @@
         <v>111</v>
       </c>
       <c r="L25">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="M25">
         <v>4</v>
       </c>
       <c r="N25">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O25">
         <v>0</v>
@@ -1963,7 +1966,7 @@
         <v>0</v>
       </c>
       <c r="Q25" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="26" spans="1:17">
@@ -2013,7 +2016,7 @@
         <v>0</v>
       </c>
       <c r="Q26" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="27" spans="1:17">
@@ -2063,7 +2066,7 @@
         <v>0</v>
       </c>
       <c r="Q27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="28" spans="1:17">
@@ -2113,7 +2116,7 @@
         <v>0</v>
       </c>
       <c r="Q28" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="29" spans="1:17">
@@ -2163,7 +2166,7 @@
         <v>0</v>
       </c>
       <c r="Q29" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="30" spans="1:17">
@@ -2213,7 +2216,7 @@
         <v>0</v>
       </c>
       <c r="Q30" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="31" spans="1:17">
@@ -2263,7 +2266,7 @@
         <v>0</v>
       </c>
       <c r="Q31" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="32" spans="1:17">
@@ -2313,7 +2316,7 @@
         <v>0</v>
       </c>
       <c r="Q32" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="33" spans="1:17">
@@ -2363,7 +2366,7 @@
         <v>0</v>
       </c>
       <c r="Q33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="34" spans="1:17">
@@ -2413,7 +2416,7 @@
         <v>0</v>
       </c>
       <c r="Q34" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="35" spans="1:17">
@@ -2463,7 +2466,7 @@
         <v>0</v>
       </c>
       <c r="Q35" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="36" spans="1:17">
@@ -2513,7 +2516,7 @@
         <v>0</v>
       </c>
       <c r="Q36" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="37" spans="1:17">
@@ -2563,7 +2566,7 @@
         <v>0</v>
       </c>
       <c r="Q37" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="38" spans="1:17">
@@ -2613,7 +2616,7 @@
         <v>0</v>
       </c>
       <c r="Q38" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="39" spans="1:17">
@@ -2663,7 +2666,7 @@
         <v>0</v>
       </c>
       <c r="Q39" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="40" spans="1:17">
@@ -2713,7 +2716,7 @@
         <v>0</v>
       </c>
       <c r="Q40" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="41" spans="1:17">
@@ -2763,7 +2766,7 @@
         <v>0</v>
       </c>
       <c r="Q41" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="42" spans="1:17">
@@ -2795,7 +2798,7 @@
         <v>115.1964986</v>
       </c>
       <c r="K42" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -2813,7 +2816,7 @@
         <v>0</v>
       </c>
       <c r="Q42" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="43" spans="1:17">
@@ -2863,7 +2866,7 @@
         <v>0</v>
       </c>
       <c r="Q43" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update INARA Beta 12 WOK 2026-10-18 08:35:30
</commit_message>
<xml_diff>
--- a/beta_12wok/detail_odp_black_special_value.xlsx
+++ b/beta_12wok/detail_odp_black_special_value.xlsx
@@ -1448,16 +1448,16 @@
         <v>116.3120566</v>
       </c>
       <c r="K15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15">
         <v>0</v>
       </c>
       <c r="N15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O15">
         <v>0</v>
@@ -1951,13 +1951,13 @@
         <v>111</v>
       </c>
       <c r="L25">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M25">
         <v>4</v>
       </c>
       <c r="N25">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O25">
         <v>0</v>

</xml_diff>

<commit_message>
Update INARA Beta 12 WOK 2026-10-21 15:52:32
</commit_message>
<xml_diff>
--- a/beta_12wok/detail_odp_black_special_value.xlsx
+++ b/beta_12wok/detail_odp_black_special_value.xlsx
@@ -2501,13 +2501,13 @@
         <v>109</v>
       </c>
       <c r="L36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M36">
         <v>1</v>
       </c>
       <c r="N36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O36">
         <v>0</v>
@@ -2698,16 +2698,16 @@
         <v>115.1955531</v>
       </c>
       <c r="K40" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M40">
         <v>0</v>
       </c>
       <c r="N40">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O40">
         <v>0</v>

</xml_diff>

<commit_message>
Update INARA Beta 12 WOK 2026-10-29 16:00:31
</commit_message>
<xml_diff>
--- a/beta_12wok/detail_odp_black_special_value.xlsx
+++ b/beta_12wok/detail_odp_black_special_value.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="113">
   <si>
     <t>ODP</t>
   </si>
@@ -347,9 +347,6 @@
   </si>
   <si>
     <t>BLACK</t>
-  </si>
-  <si>
-    <t>RED</t>
   </si>
   <si>
     <t>YELLOW</t>
@@ -816,7 +813,7 @@
         <v>0</v>
       </c>
       <c r="Q2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -866,7 +863,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -916,7 +913,7 @@
         <v>0</v>
       </c>
       <c r="Q4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:17">
@@ -966,7 +963,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -1016,7 +1013,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -1066,7 +1063,7 @@
         <v>0</v>
       </c>
       <c r="Q7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -1116,7 +1113,7 @@
         <v>0</v>
       </c>
       <c r="Q8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -1166,7 +1163,7 @@
         <v>0</v>
       </c>
       <c r="Q9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -1216,7 +1213,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:17">
@@ -1266,7 +1263,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:17">
@@ -1316,7 +1313,7 @@
         <v>0</v>
       </c>
       <c r="Q12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:17">
@@ -1366,7 +1363,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" spans="1:17">
@@ -1416,7 +1413,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:17">
@@ -1466,7 +1463,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:17">
@@ -1516,7 +1513,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="17" spans="1:17">
@@ -1566,7 +1563,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:17">
@@ -1616,7 +1613,7 @@
         <v>0</v>
       </c>
       <c r="Q18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:17">
@@ -1666,7 +1663,7 @@
         <v>0</v>
       </c>
       <c r="Q19" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:17">
@@ -1716,7 +1713,7 @@
         <v>0</v>
       </c>
       <c r="Q20" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:17">
@@ -1766,7 +1763,7 @@
         <v>0</v>
       </c>
       <c r="Q21" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:17">
@@ -1816,7 +1813,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23" spans="1:17">
@@ -1866,7 +1863,7 @@
         <v>0</v>
       </c>
       <c r="Q23" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="24" spans="1:17">
@@ -1916,7 +1913,7 @@
         <v>0</v>
       </c>
       <c r="Q24" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="25" spans="1:17">
@@ -1951,13 +1948,13 @@
         <v>111</v>
       </c>
       <c r="L25">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M25">
         <v>4</v>
       </c>
       <c r="N25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O25">
         <v>0</v>
@@ -1966,7 +1963,7 @@
         <v>0</v>
       </c>
       <c r="Q25" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="26" spans="1:17">
@@ -2016,7 +2013,7 @@
         <v>0</v>
       </c>
       <c r="Q26" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="27" spans="1:17">
@@ -2066,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="Q27" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28" spans="1:17">
@@ -2116,7 +2113,7 @@
         <v>0</v>
       </c>
       <c r="Q28" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" spans="1:17">
@@ -2166,7 +2163,7 @@
         <v>0</v>
       </c>
       <c r="Q29" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="30" spans="1:17">
@@ -2216,7 +2213,7 @@
         <v>0</v>
       </c>
       <c r="Q30" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="31" spans="1:17">
@@ -2266,7 +2263,7 @@
         <v>0</v>
       </c>
       <c r="Q31" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="32" spans="1:17">
@@ -2316,7 +2313,7 @@
         <v>0</v>
       </c>
       <c r="Q32" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="33" spans="1:17">
@@ -2366,7 +2363,7 @@
         <v>0</v>
       </c>
       <c r="Q33" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="34" spans="1:17">
@@ -2416,7 +2413,7 @@
         <v>0</v>
       </c>
       <c r="Q34" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="35" spans="1:17">
@@ -2466,7 +2463,7 @@
         <v>0</v>
       </c>
       <c r="Q35" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="36" spans="1:17">
@@ -2516,7 +2513,7 @@
         <v>0</v>
       </c>
       <c r="Q36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="37" spans="1:17">
@@ -2566,7 +2563,7 @@
         <v>0</v>
       </c>
       <c r="Q37" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="38" spans="1:17">
@@ -2616,7 +2613,7 @@
         <v>0</v>
       </c>
       <c r="Q38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="39" spans="1:17">
@@ -2666,7 +2663,7 @@
         <v>0</v>
       </c>
       <c r="Q39" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="40" spans="1:17">
@@ -2716,7 +2713,7 @@
         <v>0</v>
       </c>
       <c r="Q40" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="41" spans="1:17">
@@ -2766,7 +2763,7 @@
         <v>0</v>
       </c>
       <c r="Q41" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="42" spans="1:17">
@@ -2798,7 +2795,7 @@
         <v>115.1964986</v>
       </c>
       <c r="K42" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -2816,7 +2813,7 @@
         <v>0</v>
       </c>
       <c r="Q42" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="43" spans="1:17">
@@ -2866,7 +2863,7 @@
         <v>0</v>
       </c>
       <c r="Q43" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>